<commit_message>
FIX: Script 1 (perfiles) arreglado. Ahora extrae los datos con precisión.
</commit_message>
<xml_diff>
--- a/outputs/Perfiles.xlsx
+++ b/outputs/Perfiles.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Hoja 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$X$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$U$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X42"/>
+  <dimension ref="A1:U42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -463,19 +463,16 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
-    <col width="60" customWidth="1" min="14" max="14"/>
-    <col width="39" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="15" max="15"/>
     <col width="19" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="29" customWidth="1" min="17" max="17"/>
     <col width="49" customWidth="1" min="18" max="18"/>
     <col width="57" customWidth="1" min="19" max="19"/>
     <col width="31" customWidth="1" min="20" max="20"/>
     <col width="60" customWidth="1" min="21" max="21"/>
-    <col width="8" customWidth="1" min="22" max="22"/>
-    <col width="9" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -579,21 +576,6 @@
           <t>Casa de gestión</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Año</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Periodo</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Memorias de receso</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -654,17 +636,17 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Gestión Pública con Especialidad en Gobierno y Administración</t>
+          <t>Ciencia Política</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Gestión Pública con Especialidad en Gobierno y Administración</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Instituto Tecnológico Latinoamericano</t>
+          <t>Instituto Tecnológico Autónomo de México (ITAM)</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -674,7 +656,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.191</t>
+          <t>01 (222) 372 11 00 Ext. 191</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -684,32 +666,17 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Calle Vicente Guerrero no. 123, Colonia Centro, Xicotepec de Juárez, Puebla, C.P. 73080</t>
-        </is>
-      </c>
-      <c r="V2" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W2" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X2" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -777,7 +744,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -792,7 +759,7 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.206</t>
+          <t>01 (222) 372 11 00 Ext. 206</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -813,21 +780,6 @@
       <c r="U3" s="2" t="inlineStr">
         <is>
           <t>Calle Boulevard Bicentenario #3, Localidad Texcapa, Huauchinango, Puebla. CP 73172.</t>
-        </is>
-      </c>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W3" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X3" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -880,7 +832,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -910,7 +862,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.197</t>
+          <t>01 (222) 372 11 00 Ext. 197</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -920,32 +872,17 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
           <t>Plaza la Ensenada local 36, calle Portal Guerrero No. 1, Col. Centro Chignahuapan, Pue., C. P. 73300</t>
-        </is>
-      </c>
-      <c r="V4" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W4" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X4" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1013,7 +950,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -1028,7 +965,7 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.179</t>
+          <t>01 (222) 372 11 00 Ext. 179</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -1043,27 +980,12 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
           <t>Santos Degollado 118, Centro, Hueyapan, Puebla. C.P. 73920</t>
-        </is>
-      </c>
-      <c r="V5" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W5" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X5" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1053,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -1146,7 +1068,7 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.193</t>
+          <t>01 (222) 372 11 00 Ext. 193</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -1161,27 +1083,12 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
           <t>Calle 4 Norte #1092, Barrio de Guadalupe, Libres, Pue.</t>
-        </is>
-      </c>
-      <c r="V6" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W6" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X6" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1249,22 +1156,22 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Docente</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Universidad Pedagógica Nacional de Teziutlán</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Pública</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.195</t>
+          <t>01 (222) 372 11 00 Ext. 195</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -1279,27 +1186,12 @@
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
           <t>Calle Bicentenario #2, Colonia Centro, CP 73880, Teziutlán, Puebla.</t>
-        </is>
-      </c>
-      <c r="V7" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W7" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X7" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1259,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1382,7 +1274,7 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.185</t>
+          <t>01 (222) 372 11 00 Ext. 185</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -1392,32 +1284,17 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
           <t>Calle independencia norte #127 Colonia Centro, San Martín Texmelucan, Puebla.</t>
-        </is>
-      </c>
-      <c r="V8" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W8" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X8" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1480,27 +1357,27 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Comunicación y Medios Digitales</t>
+          <t>Ciencias de la Comunicación</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Comunicación y Medios Digitales</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>UDLAP</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.159</t>
+          <t>01 (222) 372 11 00 Ext. 159</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -1521,21 +1398,6 @@
       <c r="U9" s="2" t="inlineStr">
         <is>
           <t>Calle Emiliano Zapata #390, Cuarto Barrio, Huejotzingo, Pue. C.P. 74160</t>
-        </is>
-      </c>
-      <c r="V9" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W9" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X9" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1593,32 +1455,32 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Licenciatura</t>
+          <t>Doctorado</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Derecho</t>
+          <t>Derecho, Magna Cum Laude</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Licenciada en Derecho</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>UDLAP</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.131</t>
+          <t>01 (222) 372 11 00 Ext. 131</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
@@ -1639,21 +1501,6 @@
       <c r="U10" s="2" t="inlineStr">
         <is>
           <t>Avenida Madrid número 120, colonia Las Trojes, San Lorenzo Almecatla. C.P. 72710, Cuautlancingo, Pue.</t>
-        </is>
-      </c>
-      <c r="V10" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W10" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X10" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1711,17 +1558,17 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Licenciatura</t>
+          <t>Licenciatura (titulación en curso)</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Administración de Empresas (titulación en curso)</t>
+          <t>Administración de Empresas</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1736,7 +1583,7 @@
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.187</t>
+          <t>01 (222) 372 11 00 Ext. 187</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
@@ -1757,21 +1604,6 @@
       <c r="U11" s="2" t="inlineStr">
         <is>
           <t>Prolongación 9 norte número 10016 local 8, en la Colonia Villa Frontera de esta Ciudad de Puebla, Puebla.</t>
-        </is>
-      </c>
-      <c r="V11" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W11" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X11" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1829,32 +1661,32 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Licenciatura</t>
+          <t>Especialidad</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Relaciones Internacionales- Titulación en proceso</t>
+          <t>Relaciones Internacionales</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>BUAP</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Pública</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.160</t>
+          <t>01 (222) 372 11 00 Ext. 160</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
@@ -1875,21 +1707,6 @@
       <c r="U12" s="2" t="inlineStr">
         <is>
           <t>Calle Plazuela de San Francisco #1401 esq. Av. Tecamachalco col. Plazas Amalucan CP.72311</t>
-        </is>
-      </c>
-      <c r="V12" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W12" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X12" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1957,22 +1774,22 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>BUAP</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Pública</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.222</t>
+          <t>01 (222) 372 11 00 Ext. 222</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
@@ -1987,27 +1804,12 @@
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
           <t>Cerrada Guayacán, S/N, colonia El Arenal, Chachapa, Amozoc, Estado de Puebla</t>
-        </is>
-      </c>
-      <c r="V13" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W13" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X13" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2070,27 +1872,27 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Ciencia Política y Gestión Pública</t>
+          <t>Derecho</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Ciencia Política y Gestión Pública</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>UPAEP</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.555</t>
+          <t>01 (222) 372 11 00 Ext. 555</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
@@ -2111,21 +1913,6 @@
       <c r="U14" s="2" t="inlineStr">
         <is>
           <t>Calle Negrete Poniente, número 206 A, Colonia Centro, Tepeaca, Puebla, con Código Postal 75200.</t>
-        </is>
-      </c>
-      <c r="V14" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W14" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X14" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2188,27 +1975,27 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Investigación Educativa</t>
+          <t>Ingeniería Industrial</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Doctorado en Investigación Educativa</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Instituto Tecnológico Superior de Zacapoaxtla</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Pública</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.163</t>
+          <t>01 (222) 372 11 00 Ext. 163</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
@@ -2229,21 +2016,6 @@
       <c r="U15" s="2" t="inlineStr">
         <is>
           <t>Calle Carlos B. Zetina No. 202 Col. Centro, Ciudad Serdán Puebla.</t>
-        </is>
-      </c>
-      <c r="V15" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W15" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X15" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2301,32 +2073,32 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Maestría</t>
+          <t>Licenciatura</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Ciencias de Gobierno y Desarrollo Sustentable - En curso</t>
+          <t>Administración</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Ciencias de Gobierno y Desarrollo Sustentable - En curso</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>BUAP</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Pública</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.231</t>
+          <t>01 (222) 372 11 00 Ext. 231</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
@@ -2347,21 +2119,6 @@
       <c r="U16" s="2" t="inlineStr">
         <is>
           <t>Av. 9 poniente número 801, Col. Centro, Tecamachalco, Puebla. C. P. 75487</t>
-        </is>
-      </c>
-      <c r="V16" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W16" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X16" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2171,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -2429,22 +2186,22 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>UDLAP</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.162</t>
+          <t>01 (222) 372 11 00 Ext. 162</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
@@ -2465,21 +2222,6 @@
       <c r="U17" s="2" t="inlineStr">
         <is>
           <t>Av. Del Jardín número 2239, local 7 modulo H. planta alta del cuerpo poniente, interior de la Plaza GAALLA. Colonia Rancho San José Xilotzingo, Puebla, Pue. C. P. 72570. Teléfonos (222) 290-3884 y celular (222) 402-1112</t>
-        </is>
-      </c>
-      <c r="V17" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W17" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X17" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2542,27 +2284,27 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Psicopedagogía</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Psicopedagogía</t>
+          <t>Docente</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Universidad Madero</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.194</t>
+          <t>01 (222) 372 11 00 Ext. 194</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
@@ -2583,21 +2325,6 @@
       <c r="U18" s="2" t="inlineStr">
         <is>
           <t>Av. 32 Oriente número 202, Colonia Mártires del Trabajo, Puebla, Puebla, C.P. 72000</t>
-        </is>
-      </c>
-      <c r="V18" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W18" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X18" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2660,27 +2387,27 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Administración Pública</t>
+          <t>Ciencias de la Comunicación</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Administración Pública</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Universidad Madero</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.201</t>
+          <t>01 (222) 372 11 00 Ext. 201</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
@@ -2701,21 +2428,6 @@
       <c r="U19" s="2" t="inlineStr">
         <is>
           <t>Calle 9 Poniente 1312, La Santísima, Barrio de Santa María Xixitla, 72762 Cholula de Rivadavia, Pue.</t>
-        </is>
-      </c>
-      <c r="V19" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W19" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X19" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2783,22 +2495,22 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>IAP</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Pública</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.241</t>
+          <t>01 (222) 372 11 00 Ext. 241</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
@@ -2819,21 +2531,6 @@
       <c r="U20" s="2" t="inlineStr">
         <is>
           <t>Av. 32 Oriente número 202, Colonia Mártires del Trabajo, Puebla, Puebla, C.P. 72000</t>
-        </is>
-      </c>
-      <c r="V20" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W20" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X20" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2583,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2901,22 +2598,22 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Centro Universitario para el Desarrollo Empresarial de México</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.171</t>
+          <t>01 (222) 372 11 00 Ext. 171</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
@@ -2937,21 +2634,6 @@
       <c r="U21" s="2" t="inlineStr">
         <is>
           <t>Plaza Guadalupe, oficina 102.. Prolongación De la 16 de septiembre 12105, Guadalupe Hidalgo, C:P. 72090</t>
-        </is>
-      </c>
-      <c r="V21" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W21" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X21" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -3019,7 +2701,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
@@ -3034,7 +2716,7 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.376</t>
+          <t>01 (222) 372 11 00 Ext. 376</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
@@ -3044,32 +2726,17 @@
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
         <is>
           <t>Av. Los volcanes No. 2917 Col. El Popo, Atlixco Pue.</t>
-        </is>
-      </c>
-      <c r="V22" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W22" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X22" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -3137,22 +2804,22 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Docente</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Escuela Normal Superior del Estado de Puebla</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Pública</t>
         </is>
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.230</t>
+          <t>01 (222) 372 11 00 Ext. 230</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
@@ -3173,21 +2840,6 @@
       <c r="U23" s="2" t="inlineStr">
         <is>
           <t>Coquixtlan No. 35 Col. Los Reyes, Izúcar de Matamoros. Puebla. C. P. 74490.</t>
-        </is>
-      </c>
-      <c r="V23" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W23" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X23" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -3240,7 +2892,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -3250,27 +2902,27 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Derecho Cursado en el Instituto Mixteco de Educación Integral</t>
+          <t>Derecho</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Instituto Mixteco de Educación Integral</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.175</t>
+          <t>01 (222) 372 11 00 Ext. 175</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr">
@@ -3291,21 +2943,6 @@
       <c r="U24" s="2" t="inlineStr">
         <is>
           <t>Calle Benito Juárez No. 5, Col. San Juan, Acatlán de Osorio, Puebla. C P.74949</t>
-        </is>
-      </c>
-      <c r="V24" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W24" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X24" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -3368,27 +3005,27 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Derecho (Abogado Notario y Actuario)</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Educación</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>BUAP</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Pública</t>
         </is>
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.177</t>
+          <t>01 (222) 372 11 00 Ext. 177</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr">
@@ -3403,27 +3040,12 @@
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U25" s="2" t="inlineStr">
         <is>
           <t>Dos Casas de Gestión: Calzada Adolfo López Mateos #3210 Plaza Tehuacán local 12planta alta, Tehuacán, Puebla. La segunda Avenida Nacional número 107, colonia centro, de la junta auxiliar de San Andrés Cacaloapan, municipio de Tepanco de López.</t>
-        </is>
-      </c>
-      <c r="V25" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W25" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X25" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -3486,27 +3108,27 @@
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>Derecho en la Universidad Interamericana para el Desarrollo</t>
+          <t>Derecho</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>UNID</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.238</t>
+          <t>01 (222) 372 11 00 Ext. 238</t>
         </is>
       </c>
       <c r="R26" s="2" t="inlineStr">
@@ -3527,21 +3149,6 @@
       <c r="U26" s="2" t="inlineStr">
         <is>
           <t>20 poniente 1609, San Nicolás Tetitzintla, Tehuacán, Puebla. Cp. 75710</t>
-        </is>
-      </c>
-      <c r="V26" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W26" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X26" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -3604,27 +3211,27 @@
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Producción</t>
+          <t>Ing Industrial en Producción</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>Ingeniero Industrial En Producción</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Instituto Tecnológico De Puebla</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Pública</t>
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.148</t>
+          <t>01 (222) 372 11 00 Ext. 148</t>
         </is>
       </c>
       <c r="R27" s="2" t="inlineStr">
@@ -3634,7 +3241,7 @@
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="T27" s="2" t="inlineStr">
@@ -3645,21 +3252,6 @@
       <c r="U27" s="2" t="inlineStr">
         <is>
           <t>Av. Rafael Ávila Camacho s/n, barrio Pantzingo, Ajalpan, Pue.</t>
-        </is>
-      </c>
-      <c r="V27" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W27" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X27" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -3724,27 +3316,27 @@
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza y Gobiernos Locales</t>
+          <t>Derecho</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Gobernanza y Gobiernos Locales</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>BUAP</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Pública</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.128</t>
+          <t>01 (222) 372 11 00 Ext. 128</t>
         </is>
       </c>
       <c r="R28" s="2" t="inlineStr">
@@ -3765,21 +3357,6 @@
       <c r="U28" s="2" t="inlineStr">
         <is>
           <t>Calle Tamarindo, número 42, Colonia Arboledas de Guadalupe de esta Ciudad Capital.</t>
-        </is>
-      </c>
-      <c r="V28" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W28" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X28" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -3834,7 +3411,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -3864,7 +3441,7 @@
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.233</t>
+          <t>01 (222) 372 11 00 Ext. 233</t>
         </is>
       </c>
       <c r="R29" s="2" t="inlineStr">
@@ -3874,7 +3451,7 @@
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="T29" s="2" t="inlineStr">
@@ -3884,22 +3461,7 @@
       </c>
       <c r="U29" s="2" t="inlineStr">
         <is>
-          <t>Calle Pablo L. Sidar  número 259-E, Segundo Barrio,  Huejotzingo, Pue. C. P. 74160</t>
-        </is>
-      </c>
-      <c r="V29" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W29" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X29" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
+          <t>Calle Pablo L. Sidar número 259-E, Segundo Barrio, Huejotzingo, Pue. C. P. 74160</t>
         </is>
       </c>
     </row>
@@ -3954,7 +3516,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -3984,7 +3546,7 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.235</t>
+          <t>01 (222) 372 11 00 Ext. 235</t>
         </is>
       </c>
       <c r="R30" s="2" t="inlineStr">
@@ -4005,21 +3567,6 @@
       <c r="U30" s="2" t="inlineStr">
         <is>
           <t>Calle Mujica y Osorio #13, 3er piso, Colonia Centro, San Martín Texmelucan, Puebla</t>
-        </is>
-      </c>
-      <c r="V30" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W30" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X30" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -4089,7 +3636,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Administradora</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
@@ -4104,7 +3651,7 @@
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.234</t>
+          <t>01 (222) 372 11 00 Ext. 234</t>
         </is>
       </c>
       <c r="R31" s="2" t="inlineStr">
@@ -4114,32 +3661,17 @@
       </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U31" s="2" t="inlineStr">
         <is>
           <t>Av. 32 Oriente número 202, Colonia Mártires del Trabajo, Puebla, Puebla, C.P. 72000</t>
-        </is>
-      </c>
-      <c r="V31" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W31" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X31" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -4204,27 +3736,27 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Gobierno y Políticas Públicas</t>
+          <t>Administración Pública</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Gobierno y Políticas Públicas</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>BUAP</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Pública</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.243</t>
+          <t>01 (222) 372 11 00 Ext. 243</t>
         </is>
       </c>
       <c r="R32" s="2" t="inlineStr">
@@ -4234,32 +3766,17 @@
       </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="T32" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U32" s="2" t="inlineStr">
         <is>
           <t>Av. 32 Oriente número 202, Colonia Mártires del Trabajo, Puebla, Puebla, C.P. 72000</t>
-        </is>
-      </c>
-      <c r="V32" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W32" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X32" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -4329,7 +3846,7 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
@@ -4344,7 +3861,7 @@
       </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.309</t>
+          <t>01 (222) 372 11 00 Ext. 309</t>
         </is>
       </c>
       <c r="R33" s="2" t="inlineStr">
@@ -4354,32 +3871,17 @@
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="T33" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U33" s="2" t="inlineStr">
         <is>
           <t>Avenida Ciudad Militar No. 36, Colonia Ignacio Zaragoza, (entre Calle Pino Suárez y Niños Héroes), C.P. 72380, en Puebla, Pue.</t>
-        </is>
-      </c>
-      <c r="V33" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W33" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X33" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -4444,27 +3946,27 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>Política y Gestión Publica</t>
+          <t>Derecho</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Política y Gestión Publica</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Universidad Iberoamericana de León</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.142</t>
+          <t>01 (222) 372 11 00 Ext. 142</t>
         </is>
       </c>
       <c r="R34" s="2" t="inlineStr">
@@ -4485,21 +3987,6 @@
       <c r="U34" s="2" t="inlineStr">
         <is>
           <t>Av. Juárez número 2925, Colonia la Paz, Puebla, Puebla. CP. 72160 Piso 18. Oficina 1801</t>
-        </is>
-      </c>
-      <c r="V34" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W34" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X34" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4041,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -4564,27 +4051,27 @@
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>Ciencias Políticas Universidad Popular Autónoma del Estado de Puebla</t>
+          <t>Ciencias Políticas</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Ciencias Políticas</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>UPAEP</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.249</t>
+          <t>01 (222) 372 11 00 Ext. 249</t>
         </is>
       </c>
       <c r="R35" s="2" t="inlineStr">
@@ -4599,27 +4086,12 @@
       </c>
       <c r="T35" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U35" s="2" t="inlineStr">
         <is>
           <t>Calle Emiliano Zapata s/n C. P. 75980, entre Aristeo de la Vega y Calle La Soledad, Coxcatlán, Pue.</t>
-        </is>
-      </c>
-      <c r="V35" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W35" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X35" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -4684,27 +4156,27 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>Administración Pública</t>
+          <t>Derecho</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Administración Pública</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Universidad Nacional Autónoma de México</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Pública</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.158</t>
+          <t>01 (222) 372 11 00 Ext. 158</t>
         </is>
       </c>
       <c r="R36" s="2" t="inlineStr">
@@ -4725,21 +4197,6 @@
       <c r="U36" s="2" t="inlineStr">
         <is>
           <t>Calle 29 C Sur 3505, Col. El Vergel, C.P. 72400 Puebla, Pue</t>
-        </is>
-      </c>
-      <c r="V36" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W36" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X36" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -4809,22 +4266,22 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>UDLAP</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.161</t>
+          <t>01 (222) 372 11 00 Ext. 161</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
@@ -4845,21 +4302,6 @@
       <c r="U37" s="2" t="inlineStr">
         <is>
           <t>11 sur, esquina con 81 poniente, Col. San José Mayorazgo.</t>
-        </is>
-      </c>
-      <c r="V37" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W37" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X37" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -4929,22 +4371,22 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Político</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>UPAEP</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.165</t>
+          <t>01 (222) 372 11 00 Ext. 165</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
@@ -4965,21 +4407,6 @@
       <c r="U38" s="2" t="inlineStr">
         <is>
           <t>Planta Baja, No.22 en Avenida 32 oriente #202, Col. Mártires de Trabajo, Puebla, Puebla.</t>
-        </is>
-      </c>
-      <c r="V38" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W38" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X38" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -5034,7 +4461,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -5064,7 +4491,7 @@
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.144</t>
+          <t>01 (222) 372 11 00 Ext. 144</t>
         </is>
       </c>
       <c r="R39" s="2" t="inlineStr">
@@ -5074,32 +4501,17 @@
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="T39" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U39" s="2" t="inlineStr">
         <is>
           <t>Camino Antiguo a Cuayantla número 1403, San Bernardino Tlaxcalancingo, San Andrés Cholula, Puebla.</t>
-        </is>
-      </c>
-      <c r="V39" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W39" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X39" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -5164,27 +4576,27 @@
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>sistemas computacionales Maestría en Administración Pública</t>
+          <t>sistemas computacionales</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>Maestría en Administración Pública</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Tecnológico de Tehuacán</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Privada</t>
         </is>
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.156</t>
+          <t>01 (222) 372 11 00 Ext. 156</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -5205,21 +4617,6 @@
       <c r="U40" s="2" t="inlineStr">
         <is>
           <t>Calle Costa Rica No.2 Unidad Magisterial Chapulco, Puebla, Pue. C.P. 72590,</t>
-        </is>
-      </c>
-      <c r="V40" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W40" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X40" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -5289,7 +4686,7 @@
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr">
@@ -5304,7 +4701,7 @@
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.246</t>
+          <t>01 (222) 372 11 00 Ext. 246</t>
         </is>
       </c>
       <c r="R41" s="2" t="inlineStr">
@@ -5325,21 +4722,6 @@
       <c r="U41" s="2" t="inlineStr">
         <is>
           <t>Av. 32 Oriente número 202, Oficina 37, Colonia Mártires del Trabajo, Puebla, Puebla, C.P. 72290</t>
-        </is>
-      </c>
-      <c r="V41" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W41" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X41" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -5389,12 +4771,12 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -5424,47 +4806,32 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>Tel. (222) 372 11 00 Ext.154</t>
+          <t>01 (222) 372 11 00 Ext. 154</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>dip.elisa.limon@congresodepuebla.mx</t>
         </is>
       </c>
       <c r="S42" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="T42" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="U42" s="2" t="inlineStr">
         <is>
           <t>Av. 5 de Mayo Sur número 505 Piso 3 interior 1, colonia Centro, Zacapoaxtla Puebla. C. P. 73680</t>
-        </is>
-      </c>
-      <c r="V42" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W42" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X42" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X42"/>
+  <autoFilter ref="A1:U42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>